<commit_message>
optimization seems to work!
</commit_message>
<xml_diff>
--- a/Results/pam_parametrizer_diagnostics.xlsx
+++ b/Results/pam_parametrizer_diagnostics.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="16">
   <si>
     <t>run_id</t>
   </si>
@@ -45,9 +45,6 @@
     <t>E5</t>
   </si>
   <si>
-    <t>E3</t>
-  </si>
-  <si>
     <t>R1</t>
   </si>
   <si>
@@ -58,9 +55,6 @@
   </si>
   <si>
     <t>R5</t>
-  </si>
-  <si>
-    <t>R3</t>
   </si>
   <si>
     <t>time_s</t>
@@ -427,7 +421,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -455,13 +449,13 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>0.8234795527161617</v>
       </c>
       <c r="E2">
-        <v>0.8705275686685858</v>
+        <v>0.8784969100006801</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -472,13 +466,13 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D3">
-        <v>1.259824996726642</v>
+        <v>0.9919446539425778</v>
       </c>
       <c r="E3">
-        <v>0.8705275686685858</v>
+        <v>0.8784969100006801</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -489,13 +483,13 @@
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4">
-        <v>0.5000000000000001</v>
+        <v>0.07380142744652554</v>
       </c>
       <c r="E4">
-        <v>0.8705275686685858</v>
+        <v>0.8784969100006801</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -506,13 +500,13 @@
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D5">
-        <v>0.6132770754758511</v>
+        <v>0.6609748738326033</v>
       </c>
       <c r="E5">
-        <v>0.8705275686685858</v>
+        <v>0.8784969100006801</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -523,13 +517,13 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D6">
-        <v>0.8777086025970818</v>
+        <v>0.8234795527161617</v>
       </c>
       <c r="E6">
-        <v>0.8713734315405167</v>
+        <v>0.8784969100006801</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -540,13 +534,13 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D7">
-        <v>1.259824996726642</v>
+        <v>0.9919446539425778</v>
       </c>
       <c r="E7">
-        <v>0.8713734315405167</v>
+        <v>0.8784969100006801</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -554,16 +548,16 @@
         <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D8">
-        <v>1.076131060133354</v>
+        <v>0.07380142744652554</v>
       </c>
       <c r="E8">
-        <v>0.8713734315405167</v>
+        <v>0.8784969100006801</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -571,16 +565,16 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C9" t="s">
         <v>12</v>
       </c>
       <c r="D9">
-        <v>0.5000000000000001</v>
+        <v>0.6609748738326033</v>
       </c>
       <c r="E9">
-        <v>0.8713734315405167</v>
+        <v>0.8784969100006801</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -591,13 +585,13 @@
         <v>5</v>
       </c>
       <c r="C10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D10">
-        <v>0.8777086025970818</v>
+        <v>0.8234795527161617</v>
       </c>
       <c r="E10">
-        <v>0.8755345448971104</v>
+        <v>0.8784969100006801</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -608,13 +602,13 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D11">
-        <v>1.259824996726642</v>
+        <v>0.9919446539425778</v>
       </c>
       <c r="E11">
-        <v>0.8755345448971104</v>
+        <v>0.8784969100006801</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -622,16 +616,16 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C12" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D12">
-        <v>1.306074582571766</v>
+        <v>0.07380142744652554</v>
       </c>
       <c r="E12">
-        <v>0.8755345448971104</v>
+        <v>0.8784969100006801</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -639,16 +633,16 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C13" t="s">
         <v>12</v>
       </c>
       <c r="D13">
-        <v>0.5000000000000001</v>
+        <v>0.6609748738326033</v>
       </c>
       <c r="E13">
-        <v>0.8755345448971104</v>
+        <v>0.8784969100006801</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -659,13 +653,13 @@
         <v>5</v>
       </c>
       <c r="C14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D14">
-        <v>0.7703723910729221</v>
+        <v>0.8234795527161617</v>
       </c>
       <c r="E14">
-        <v>0.8774400720735906</v>
+        <v>0.8784969383669554</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -676,13 +670,13 @@
         <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D15">
-        <v>1.437910246689462</v>
+        <v>1.902231809966862</v>
       </c>
       <c r="E15">
-        <v>0.8774400720735906</v>
+        <v>0.8784969383669554</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -690,16 +684,16 @@
         <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C16" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D16">
-        <v>1.405507425156182</v>
+        <v>0.05228343228324275</v>
       </c>
       <c r="E16">
-        <v>0.8774400720735906</v>
+        <v>0.8784969383669554</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -707,16 +701,492 @@
         <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C17" t="s">
         <v>12</v>
       </c>
       <c r="D17">
-        <v>0.0582239853154774</v>
+        <v>0.8788668275153635</v>
       </c>
       <c r="E17">
-        <v>0.8774400720735906</v>
+        <v>0.8784969383669554</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18">
+        <v>5</v>
+      </c>
+      <c r="B18" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18">
+        <v>0.8234795527161617</v>
+      </c>
+      <c r="E18">
+        <v>0.8784969383669554</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19">
+        <v>5</v>
+      </c>
+      <c r="B19" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19">
+        <v>1.902231809966862</v>
+      </c>
+      <c r="E19">
+        <v>0.8784969383669554</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20">
+        <v>5</v>
+      </c>
+      <c r="B20" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20">
+        <v>0.05228343228324275</v>
+      </c>
+      <c r="E20">
+        <v>0.8784969383669554</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21">
+        <v>5</v>
+      </c>
+      <c r="B21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21">
+        <v>0.8788668275153635</v>
+      </c>
+      <c r="E21">
+        <v>0.8784969383669554</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22">
+        <v>6</v>
+      </c>
+      <c r="B22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C22" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22">
+        <v>0.8234795527161617</v>
+      </c>
+      <c r="E22">
+        <v>0.8784969383669554</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23">
+        <v>6</v>
+      </c>
+      <c r="B23" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23">
+        <v>1.902231809966862</v>
+      </c>
+      <c r="E23">
+        <v>0.8784969383669554</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24">
+        <v>6</v>
+      </c>
+      <c r="B24" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24">
+        <v>0.05228343228324275</v>
+      </c>
+      <c r="E24">
+        <v>0.8784969383669554</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25">
+        <v>6</v>
+      </c>
+      <c r="B25" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25">
+        <v>0.8788668275153635</v>
+      </c>
+      <c r="E25">
+        <v>0.8784969383669554</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26">
+        <v>7</v>
+      </c>
+      <c r="B26" t="s">
+        <v>5</v>
+      </c>
+      <c r="C26" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26">
+        <v>0.8234795527161617</v>
+      </c>
+      <c r="E26">
+        <v>0.8784969383669552</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27">
+        <v>7</v>
+      </c>
+      <c r="B27" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27">
+        <v>1.902231809966862</v>
+      </c>
+      <c r="E27">
+        <v>0.8784969383669552</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28">
+        <v>7</v>
+      </c>
+      <c r="B28" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" t="s">
+        <v>11</v>
+      </c>
+      <c r="D28">
+        <v>0.05228343228324275</v>
+      </c>
+      <c r="E28">
+        <v>0.8784969383669552</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29">
+        <v>7</v>
+      </c>
+      <c r="B29" t="s">
+        <v>8</v>
+      </c>
+      <c r="C29" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29">
+        <v>0.8788668275153635</v>
+      </c>
+      <c r="E29">
+        <v>0.8784969383669552</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30">
+        <v>8</v>
+      </c>
+      <c r="B30" t="s">
+        <v>5</v>
+      </c>
+      <c r="C30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30">
+        <v>0.8234795527161617</v>
+      </c>
+      <c r="E30">
+        <v>0.8784969383669552</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31">
+        <v>8</v>
+      </c>
+      <c r="B31" t="s">
+        <v>6</v>
+      </c>
+      <c r="C31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31">
+        <v>1.902231809966862</v>
+      </c>
+      <c r="E31">
+        <v>0.8784969383669552</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32">
+        <v>8</v>
+      </c>
+      <c r="B32" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" t="s">
+        <v>11</v>
+      </c>
+      <c r="D32">
+        <v>0.05228343228324275</v>
+      </c>
+      <c r="E32">
+        <v>0.8784969383669552</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33">
+        <v>8</v>
+      </c>
+      <c r="B33" t="s">
+        <v>8</v>
+      </c>
+      <c r="C33" t="s">
+        <v>12</v>
+      </c>
+      <c r="D33">
+        <v>0.8788668275153635</v>
+      </c>
+      <c r="E33">
+        <v>0.8784969383669552</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34">
+        <v>9</v>
+      </c>
+      <c r="B34" t="s">
+        <v>5</v>
+      </c>
+      <c r="C34" t="s">
+        <v>9</v>
+      </c>
+      <c r="D34">
+        <v>0.8234795527161617</v>
+      </c>
+      <c r="E34">
+        <v>0.8784969383669552</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35">
+        <v>9</v>
+      </c>
+      <c r="B35" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" t="s">
+        <v>10</v>
+      </c>
+      <c r="D35">
+        <v>1.902231809966862</v>
+      </c>
+      <c r="E35">
+        <v>0.8784969383669552</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36">
+        <v>9</v>
+      </c>
+      <c r="B36" t="s">
+        <v>7</v>
+      </c>
+      <c r="C36" t="s">
+        <v>11</v>
+      </c>
+      <c r="D36">
+        <v>0.05228343228324275</v>
+      </c>
+      <c r="E36">
+        <v>0.8784969383669552</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37">
+        <v>9</v>
+      </c>
+      <c r="B37" t="s">
+        <v>8</v>
+      </c>
+      <c r="C37" t="s">
+        <v>12</v>
+      </c>
+      <c r="D37">
+        <v>0.8788668275153635</v>
+      </c>
+      <c r="E37">
+        <v>0.8784969383669552</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38">
+        <v>10</v>
+      </c>
+      <c r="B38" t="s">
+        <v>5</v>
+      </c>
+      <c r="C38" t="s">
+        <v>9</v>
+      </c>
+      <c r="D38">
+        <v>0.8234795527161617</v>
+      </c>
+      <c r="E38">
+        <v>0.8784969383669554</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="A39">
+        <v>10</v>
+      </c>
+      <c r="B39" t="s">
+        <v>6</v>
+      </c>
+      <c r="C39" t="s">
+        <v>10</v>
+      </c>
+      <c r="D39">
+        <v>1.902231809966862</v>
+      </c>
+      <c r="E39">
+        <v>0.8784969383669554</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40">
+        <v>10</v>
+      </c>
+      <c r="B40" t="s">
+        <v>7</v>
+      </c>
+      <c r="C40" t="s">
+        <v>11</v>
+      </c>
+      <c r="D40">
+        <v>0.05228343228324275</v>
+      </c>
+      <c r="E40">
+        <v>0.8784969383669554</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41">
+        <v>10</v>
+      </c>
+      <c r="B41" t="s">
+        <v>8</v>
+      </c>
+      <c r="C41" t="s">
+        <v>12</v>
+      </c>
+      <c r="D41">
+        <v>0.8788668275153635</v>
+      </c>
+      <c r="E41">
+        <v>0.8784969383669554</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42">
+        <v>11</v>
+      </c>
+      <c r="B42" t="s">
+        <v>5</v>
+      </c>
+      <c r="C42" t="s">
+        <v>9</v>
+      </c>
+      <c r="D42">
+        <v>0.8234795527161617</v>
+      </c>
+      <c r="E42">
+        <v>0.8784969383669552</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43">
+        <v>11</v>
+      </c>
+      <c r="B43" t="s">
+        <v>6</v>
+      </c>
+      <c r="C43" t="s">
+        <v>10</v>
+      </c>
+      <c r="D43">
+        <v>1.902231809966862</v>
+      </c>
+      <c r="E43">
+        <v>0.8784969383669552</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44">
+        <v>11</v>
+      </c>
+      <c r="B44" t="s">
+        <v>7</v>
+      </c>
+      <c r="C44" t="s">
+        <v>11</v>
+      </c>
+      <c r="D44">
+        <v>0.05228343228324275</v>
+      </c>
+      <c r="E44">
+        <v>0.8784969383669552</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45">
+        <v>11</v>
+      </c>
+      <c r="B45" t="s">
+        <v>8</v>
+      </c>
+      <c r="C45" t="s">
+        <v>12</v>
+      </c>
+      <c r="D45">
+        <v>0.8788668275153635</v>
+      </c>
+      <c r="E45">
+        <v>0.8784969383669552</v>
       </c>
     </row>
   </sheetData>
@@ -726,7 +1196,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -734,10 +1204,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -745,10 +1215,10 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>29.87103897600173</v>
+        <v>104.1295789340002</v>
       </c>
       <c r="C2">
-        <v>0.008297510826667147</v>
+        <v>0.02892488303722227</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -756,10 +1226,10 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>27.88222122499792</v>
+        <v>102.7108157080002</v>
       </c>
       <c r="C3">
-        <v>0.007745061451388311</v>
+        <v>0.02853078214111116</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -767,10 +1237,10 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>31.93261593400166</v>
+        <v>100.4317268140003</v>
       </c>
       <c r="C4">
-        <v>0.00887017109277824</v>
+        <v>0.02789770189277786</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -778,10 +1248,87 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>30.77415381300307</v>
+        <v>97.39032089199827</v>
       </c>
       <c r="C5">
-        <v>0.008548376059167518</v>
+        <v>0.02705286691444396</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>110.5334291479994</v>
+      </c>
+      <c r="C6">
+        <v>0.03070373031888873</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>96.75803283299683</v>
+      </c>
+      <c r="C7">
+        <v>0.02687723134249912</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>110.6610748769999</v>
+      </c>
+      <c r="C8">
+        <v>0.03073918746583331</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>110.9500694939998</v>
+      </c>
+      <c r="C9">
+        <v>0.03081946374833327</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>99.85909855499995</v>
+      </c>
+      <c r="C10">
+        <v>0.02773863848749998</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>114.1265538110019</v>
+      </c>
+      <c r="C11">
+        <v>0.0317018205030561</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>108.6280499160021</v>
+      </c>
+      <c r="C12">
+        <v>0.03017445831000057</v>
       </c>
     </row>
   </sheetData>
@@ -791,7 +1338,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -799,7 +1346,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -807,7 +1354,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>0.5812464386749968</v>
+        <v>0.8478633866255989</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -815,7 +1362,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>0.5812464386749967</v>
+        <v>0.8478633866255989</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -823,7 +1370,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>0.5812464386749967</v>
+        <v>0.8478633866255989</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -831,7 +1378,63 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>0.8459466444987327</v>
+        <v>0.847869591513823</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>0.847869591513823</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>0.847869591513823</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>0.847869591513823</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>0.847869591513823</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>0.847869591513823</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>0.847869591513823</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>0.847869591513823</v>
       </c>
     </row>
   </sheetData>

</xml_diff>